<commit_message>
Train_results_R0: add analyses A-E (init-vs-final PC, change outcomes, phase productivity, cost, failure trajectory)
Append five analyses below the spacer in the R0 table/xlsx, all computed from
experiments/subset_train-r0 (attempts.jsonl + per-query checkpoints):
 A: initial vs final personal-constraint satisfaction (improved/same/worse)
 B: mutually-exclusive change outcomes (no change / fix / regression / neutral)
 C: personal vs commonsense phase productivity
 D: cost (tokens, model calls, repair time per query)
 E: a real fix-and-regress trajectory with readable constraint families
No summary in the notebook or xlsx.
</commit_message>
<xml_diff>
--- a/train_result_analysis/Train_results_R0.xlsx
+++ b/train_result_analysis/Train_results_R0.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -560,6 +560,264 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>[A] Queries where final PC improved vs initial</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>5 / 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>[A] Queries unchanged (final PC == initial)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>47 / 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>[A] Queries where final PC worsened vs initial</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>8 / 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>[A] Net personal constraints gained (sum of deltas)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>-13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>[B] Attempts: confirmed no change (0 slots)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>198 (59.8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>[B] Attempts: change not measurable</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>46 (13.9%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>[B] Attempts: changed &amp; fixed &gt;=1 (no regression)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11 (3.3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>[B] Attempts: changed &amp; introduced a regression</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>16 (4.8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>[B] Attempts: changed but neither fixed nor regressed</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>60 (18.1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>[C] Personal attempts (count)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>[C] Personal: fixed &gt;=1 targeted constraint</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14/187 (7.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>[C] Personal: introduced a new violation</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2/187 (1.1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>[C] Personal: no confirmed change</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>169/187 (90.4%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>[C] Commonsense attempts (count)</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>[C] Commonsense: fixed &gt;=1 targeted constraint</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0/144 (0.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>[C] Commonsense: introduced a new violation</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15/144 (10.4%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>[C] Commonsense: no confirmed change</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>75/144 (52.1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>[D] Queries with complete token data</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>55 / 59</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>[D] Avg tokens per query (complete-data queries)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>96,849</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>[D] Avg model calls per query</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>[D] Avg repair time per query (s)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>96.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>[E] Example fix-and-regress trajectory</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>query e20241028160908981620, step 1 (personal): fixed monetary_budget; newly violated trip_specification</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Train_results_R0: focused 3-column table (Category | Metric | R0 TRAIN result)
Restructure the R0 train-results table into Category | Metric | value with
plain-English metric names and no summary.

Above the spacer: the common-core rows (shared by every strategy). Below the
spacer, keep a focused set of R0 insights:
- Final outcome: queries improved / unchanged / worsened, net PC gained
- Repair behaviour: confirmed no change, changed & fixed >=1 (no regression),
  changed & introduced a regression
- Efficiency: average tokens per query (stored as a number, #,##0 format),
  average repair time per query

Phase breakdown, the example fix-and-regress trajectory, and the mechanism
metrics are computed and printed in the notebook for context but kept out of
the table to keep it concise.
</commit_message>
<xml_diff>
--- a/train_result_analysis/Train_results_R0.xlsx
+++ b/train_result_analysis/Train_results_R0.xlsx
@@ -49,9 +49,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,72 +424,103 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>R0 training result</t>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>R0 TRAIN result</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Queries</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Queries evaluated</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>60</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Repair attempts</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total repair attempts</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>331</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Personal repair attempts</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Personal-constraint repair attempts</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>187</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
           <t>Commonsense repair attempts</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" s="4" t="n">
         <v>144</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Confirmed unchanged attempts</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Attempts that left the plan unchanged</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>222 (67.07%)</t>
         </is>
@@ -491,330 +529,184 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Personal constraint fixes</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Personal constraints fixed (across attempts)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Personal regressions</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Personal constraints newly broken (across attempts)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Plan-scope proposals (always whole-plan)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>331 / 331 (100.0%)</t>
+          <t>Final outcome</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Queries improved</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>5/60 (8.3%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Proposals changing &gt;=4 slots</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>53 / 285 (18.6%)</t>
+          <t>Final outcome</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Queries unchanged</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>47/60 (78.3%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Attempts with multiple declared personal targets</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>36 / 331 (10.9%)</t>
+          <t>Final outcome</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Queries worsened</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>8/60 (13.3%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Commonsense proposals that regressed a personal constraint</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>15 / 144 (10.4%)</t>
-        </is>
+          <t>Final outcome</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Net personal constraints gained</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>-13</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>[A] Queries where final PC improved vs initial</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>5 / 60</t>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Attempts with confirmed no change</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>198/331 (59.8%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>[A] Queries unchanged (final PC == initial)</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>47 / 60</t>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Changed and fixed ≥1 without regression</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>11/331 (3.3%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>[A] Queries where final PC worsened vs initial</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>8 / 60</t>
+          <t>Repair behaviour</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Changed and introduced a regression</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>16/331 (4.8%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>[A] Net personal constraints gained (sum of deltas)</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>-13</v>
+          <t>Efficiency</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Average tokens per query</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>96849</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>[B] Attempts: confirmed no change (0 slots)</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>198 (59.8%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>[B] Attempts: change not measurable</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>46 (13.9%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>[B] Attempts: changed &amp; fixed &gt;=1 (no regression)</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>11 (3.3%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>[B] Attempts: changed &amp; introduced a regression</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>16 (4.8%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>[B] Attempts: changed but neither fixed nor regressed</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>60 (18.1%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>[C] Personal attempts (count)</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>[C] Personal: fixed &gt;=1 targeted constraint</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>14/187 (7.5%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>[C] Personal: introduced a new violation</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>2/187 (1.1%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>[C] Personal: no confirmed change</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>169/187 (90.4%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>[C] Commonsense attempts (count)</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>[C] Commonsense: fixed &gt;=1 targeted constraint</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>0/144 (0.0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>[C] Commonsense: introduced a new violation</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>15/144 (10.4%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>[C] Commonsense: no confirmed change</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>75/144 (52.1%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>[D] Queries with complete token data</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>55 / 59</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>[D] Avg tokens per query (complete-data queries)</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>96,849</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>[D] Avg model calls per query</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>2.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>[D] Avg repair time per query (s)</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>96.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>[E] Example fix-and-regress trajectory</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>query e20241028160908981620, step 1 (personal): fixed monetary_budget; newly violated trip_specification</t>
+          <t>Efficiency</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Average repair time per query</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>96.0 s</t>
         </is>
       </c>
     </row>

</xml_diff>